<commit_message>
ETSI, CEN, CENELEC Newsrooms added for fetching
</commit_message>
<xml_diff>
--- a/Newsroom_report.xlsx
+++ b/Newsroom_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="540" windowWidth="28800" windowHeight="16500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Feed Architecture" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Resource Links" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Sources → Feeds Mapping" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="1. Feed Architecture" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2. Resource Links" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3. Sources → Feeds Mapping" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1698,7 +1698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3157,6 +3157,126 @@
       </c>
       <c r="H40" s="7" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>etsi-newsroom</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ETSI Newsroom</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>html-scrape</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>global, eu, standard, conformity</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>All Sectors</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>artificial intelligence</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>European Telecommunications Standards Institute</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>oecd-newsroom</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>OECD News — Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>html-scrape</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>global, international, policy, ai</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>All Sectors</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>artificial intelligence</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Pre-filtered OECD AI news search</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>cen-cenelec-news</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CEN-CENELEC News &amp; Events</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>html-scrape</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>global, eu, standard, conformity</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>All Sectors</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>artificial intelligence, standards</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>European standards organizations newsroom</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>